<commit_message>
Team Principal: end of season (gauges, contracts, retirements, review)
At the end of a season every team earns $ by rank (4 down to 1), gets its
prestige recomputed from its whole team-family history plus brand and last
result, and its confidence updated (title, above/below the previous rank,
no dismissal). Team families come from the new Teams_Family sheet, with
titles counted exactly per year and wins/races prorated on the family's
years (script/load_team_families_in_json.py -> data/team_families.json).

Engineer contracts run down: a renewal (same negotiation) is offered during
the last season of a contract unless the engineer retires, otherwise he is
released; retirees leave their position empty; AI teams renew and fill empty
positions with a simple rule. A season review is shown once in Team
Management.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/team_default.xlsx
+++ b/data/source/team_default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/76929c7f1b9de68b/Documents/Dada/data/source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="294" documentId="11_8F20ED55937C482908FC15CAFFAB6FCF8E869301" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE6D72E4-4779-4D68-BD84-9412AA951153}"/>
+  <xr:revisionPtr revIDLastSave="307" documentId="11_8F20ED55937C482908FC15CAFFAB6FCF8E869301" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65D0346E-1EDB-4418-B99A-87CA0BADF2F0}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -693,7 +693,7 @@
         <v>44</v>
       </c>
       <c r="J4">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K4">
         <v>10</v>
@@ -763,7 +763,7 @@
         <v>42</v>
       </c>
       <c r="J6">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -798,7 +798,7 @@
         <v>45</v>
       </c>
       <c r="J7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K7">
         <v>5</v>
@@ -833,7 +833,7 @@
         <v>42</v>
       </c>
       <c r="J8">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K8">
         <v>9</v>
@@ -868,7 +868,7 @@
         <v>46</v>
       </c>
       <c r="J9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -903,7 +903,7 @@
         <v>43</v>
       </c>
       <c r="J10">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K10">
         <v>9</v>
@@ -973,7 +973,7 @@
         <v>46</v>
       </c>
       <c r="J12">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K12">
         <v>8</v>

</xml_diff>